<commit_message>
feat(F-NAR-019): ATOM-EMO.GES.002-06 Mila souffle et fait une pause
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.GES.002-06.xlsx
+++ b/stories/arbres/ATOM-EMO.GES.002-06.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La petite tour de Sarah</t>
+          <t>Mila souffle et fait une pause</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>chambre</t>
+          <t>maison, chambre, étagère, bois, fenêtre, rayon, cire, panier, cubes, tour</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sarah, papa, maman</t>
+          <t>Mila, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sarah veut une tour, puis un puzzle. Ça tombe, ça résiste. Elle souffle, fait une pause, puis reprend.</t>
+          <t>Le bois de l'étagère sent la cire. Près du bord, un éclat d'étagère brille. Mila veut la tour, maintenant. Les cubes glissent. La tour tombe. Épaules serrées, sourire parti, maman accroupie. Elle souffle, pause. Merci vécu. Cube derrière l'étagère, trop vite. Elle s'arrête, lit l'éclat. Un éclat d'étagère tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la lampe ronde allume le tapis. Un cercle de lumière, tout chaud. Des chaussettes sèchent sur le radiateur. Elles sentent encore un peu le savon. Une boîte de puzzle est ouverte, près du lit. Des pièces colorées attendent sur le bois. Je plie un pull, Sarah. J'apporte un verre d'eau. La chambre sent le linge propre. Le tapis est doux sous les pieds. Je veux une tour, maman. Les cubes sont dans le panier. On reste un moment, ensemble. En ce moment, Sarah s'assoit sous la lampe. Elle prend des cubes, un par un. Les cubes sont lisses, un peu froids. Elle pose un cube. Puis un autre. Tu montes tout doucement ? Oui. Très haut. Les cubes glissent. La tour tombe. Les épaules de Sarah se serrent. Sa poitrine va trop vite. C'est trop. Je suis fâchée. La tour est tombée. Tu es fâchée. On peut souffler. On peut faire une pause. Sarah s'assoit sur le tapis. Elle pose les mains sur ses genoux. Elle souffle une fois. Elle souffle encore. Elle fait une pause. La pause dure un moment. La lampe reste ronde et calme. Je souffle. Je fais une pause. Bravo. Tes épaules redescendent. Tu as soufflé. Tu as fait une pause. Tu veux reprendre, tout doucement ? Oui. Un cube, puis un autre. Sarah reprend les cubes. Elle pose un cube, puis un autre. La tour tient.</t>
+          <t>Le bois de l'étagère sent la cire. Ça sent le bois, un peu. Ça sent bon, papa. Tu le sens, le bois, Mila ? Oui, papa. Un rayon glisse sur le bord. Il brille, maman. Le bois est chaud ? Un peu, maman. Les cubes attendent, dans le panier. Oui, maman. Un fil de poussière danse près du bois. Il vole, papa. Tu le vois, le fil ? Oui. Le panier est lisse contre les doigts. Il est froid, maman. Tu le sens, le panier ? Oui. Près du bord, un éclat d'étagère brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Une poussière dore au-dessus du bois. Elle dore, maman. Au-dessus du bord ? Oui, au-dessus. Mila pose les mains sur le panier. Les cubes sont un peu froids. On fait la tour, papa ? Tu veux la tour, Mila ? Oui, une tour. Les cubes tapent le bois. C'est dur, papa. Comme une maison ? Oui, comme une maison. En ce moment, Mila tire le panier vers le bois. Je veux la tour, maintenant ! La tour, tout de suite. Tu vois les cubes, Mila ? Oui, papa. Mila pose un cube, trop vite. Puis un autre, trop haut. Les cubes glissent. La tour tombe. Oh. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules se serrent. Elle est tombée, Mila ? Oui, papa. Tes lèvres sont serrées, Mila ? Un peu, maman. L'éclat d'étagère tremble, puis tient. Les cubes restent au sol, mêlés. C'est trop, maman. Maman s'accroupit à la même hauteur. Mila regarde maman.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la lampe ronde allume le tapis. Un cercle de lumière, tout chaud. Des chaussettes sèchent sur le radiateur. Elles sentent encore un peu le savon. Une boîte de puzzle est ouverte, près du lit. Des pièces colorées attendent sur le bois. Je plie un pull, Sarah. J'apporte un verre d'eau. La chambre sent le linge propre. Le tapis est doux sous les pieds. Je veux une tour, maman. Les cubes sont dans le panier. On reste un moment, ensemble. En ce moment, Sarah s'assoit sous la lampe. Elle prend des cubes, un par un. Les cubes sont lisses, un peu froids. Elle pose un cube. Puis un autre. Tu montes tout doucement ? Oui. Très haut. Les cubes glissent. La tour tombe. Les épaules de Sarah se serrent. Sa poitrine va trop vite. C'est trop. Je suis fâchée. La tour est tombée. Tu es fâchée. On peut souffler. On peut faire une pause. Sarah s'assoit sur le tapis. Elle pose les mains sur ses genoux. Elle souffle une fois. Elle souffle encore. Elle fait une pause. La pause dure un moment. La lampe reste ronde et calme. Je souffle. Je fais une pause. Bravo. Tes épaules redescendent. Tu as soufflé. Tu as fait une pause. Tu veux reprendre, tout doucement ? Oui. Un cube, puis un autre. Sarah reprend les cubes. Elle pose un cube, puis un autre. La tour tient.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le bois de l'étagère sent la cire. Ça sent le bois, un peu. Ça sent bon, papa. Tu le sens, le bois, Mila ? Oui, papa. Un rayon glisse sur le bord. Il brille, maman. Le bois est chaud ? Un peu, maman. Les cubes attendent, dans le panier. Oui, maman. Un fil de poussière danse près du bois. Il vole, papa. Tu le vois, le fil ? Oui. Le panier est lisse contre les doigts. Il est froid, maman. Tu le sens, le panier ? Oui. Près du bord, un &lt;emphasis level="moderate"&gt;éclat d'étagère&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Une poussière dore au-dessus du bois. Elle dore, maman. Au-dessus du bord ? Oui, au-dessus. Mila pose les mains sur le panier. Les cubes sont un peu froids. On fait la tour, papa ? Tu veux la tour, Mila ? Oui, une tour. Les cubes tapent le bois. C'est dur, papa. Comme une maison ? Oui, comme une maison. En ce moment, Mila tire le panier vers le bois. Je veux la tour, maintenant ! La tour, tout de suite. Tu vois les cubes, Mila ? Oui, papa. Mila pose un cube, trop vite. Puis un autre, trop haut. Les cubes glissent. La tour tombe. Oh. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules se serrent. Elle est tombée, Mila ? Oui, papa. Tes lèvres sont serrées, Mila ? Un peu, maman. L'éclat d'étagère tremble, puis tient. Les cubes restent au sol, mêlés. C'est trop, maman. Maman s'accroupit à la même hauteur. Mila regarde maman.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Flore construit une tour dans sa chambre. Les cubes glissent. La tour tombe. Les épaules de Flore se serrent. Maman est près de la porte. Elle dit : on peut &lt;emphasis&gt;souffler&lt;/emphasis&gt;. On peut faire une pause. Flore s'assoit sur le tapis. Elle souffle une fois. Elle souffle encore. La pause dure un moment. Les mains se posent sur les genoux. Flore dit : je souffle. Je fais une pause. Maman hoche la tête. Puis Flore reprend les cubes. Elle pose un cube, puis un autre. La tour tient. Plus tard, un puzzle résiste. Flore se souvient. Elle s'assoit. Elle souffle. Elle fait une pause. Ensuite elle reprend. Maman sourit. [pause]</t>
+          <t>Le bois de l'étagère sent la cire. Ça sent le bois, un peu. Ça sent bon, papa. Tu le sens, le bois, Mila ? Oui, papa. Un rayon glisse sur le bord. Il brille, maman. Le bois est chaud ? Un peu, maman. Les cubes attendent, dans le panier. Oui, maman. Un fil de poussière danse près du bois. Il vole, papa. Tu le vois, le fil ? Oui. Le panier est lisse contre les doigts. Il est froid, maman. Tu le sens, le panier ? Oui. Près du bord, un &lt;emphasis&gt;éclat d'étagère&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Une poussière dore au-dessus du bois. Elle dore, maman. Au-dessus du bord ? Oui, au-dessus. Mila pose les mains sur le panier. Les cubes sont un peu froids. On fait la tour, papa ? Tu veux la tour, Mila ? Oui, une tour. Les cubes tapent le bois. C'est dur, papa. Comme une maison ? Oui, comme une maison. En ce moment, Mila tire le panier vers le bois. Je veux la tour, maintenant ! La tour, tout de suite. Tu vois les cubes, Mila ? Oui, papa. Mila pose un cube, trop vite. Puis un autre, trop haut. Les cubes glissent. La tour tombe. Oh. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules se serrent. Elle est tombée, Mila ? Oui, papa. Tes lèvres sont serrées, Mila ? Un peu, maman. L'éclat d'étagère tremble, puis tient. Les cubes restent au sol, mêlés. C'est trop, maman. Maman s'accroupit à la même hauteur. Mila regarde maman. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
         <v>1.12</v>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>souffler</t>
+          <t>éclat d'étagère</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,52 +1321,71 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis gêne; intensite=2; destinataire=enfant; sous_texte=elle_veut_la_tour_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le soir, la lampe ronde allume le tapis.
-narrateur|Un cercle de lumière, tout chaud.
-narrateur|Des chaussettes sèchent sur le radiateur.
-narrateur|Elles sentent encore un peu le savon.
-narrateur|Une boîte de puzzle est ouverte, près du lit.
-narrateur|Des pièces colorées attendent sur le bois.
-maman|Je plie un pull, Sarah.
-papa|J'apporte un verre d'eau.
-maman|La chambre sent le linge propre.
-papa|Le tapis est doux sous les pieds.
-enfant-f|Je veux une tour, maman.
-maman|Les cubes sont dans le panier.
-papa|On reste un moment, ensemble.
-narrateur|En ce moment, Sarah s'assoit sous la lampe.
-narrateur|Elle prend des cubes, un par un.
-narrateur|Les cubes sont lisses, un peu froids.
-narrateur|Elle pose un cube.
-narrateur|Puis un autre.
-papa|Tu montes tout doucement ?
-enfant-f|Oui. Très haut.
+          <t>narrateur|Le bois de l'étagère sent la cire.
+narrateur|Ça sent le bois, un peu.
+enfant-f|Ça sent bon, papa.
+papa|Tu le sens, le bois, Mila ?
+enfant-f|Oui, papa.
+narrateur|Un rayon glisse sur le bord.
+enfant-f|Il brille, maman.
+maman|Le bois est chaud ?
+enfant-f|Un peu, maman.
+maman|Les cubes attendent, dans le panier.
+enfant-f|Oui, maman.
+narrateur|Un fil de poussière danse près du bois.
+enfant-f|Il vole, papa.
+papa|Tu le vois, le fil ?
+enfant-f|Oui.
+narrateur|Le panier est lisse contre les doigts.
+enfant-f|Il est froid, maman.
+maman|Tu le sens, le panier ?
+enfant-f|Oui.
+narrateur|Près du bord, un éclat d'étagère brille.
+enfant-f|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-f|Oui, un petit point.
+narrateur|Une poussière dore au-dessus du bois.
+enfant-f|Elle dore, maman.
+maman|Au-dessus du bord ?
+enfant-f|Oui, au-dessus.
+narrateur|Mila pose les mains sur le panier.
+narrateur|Les cubes sont un peu froids.
+enfant-f|On fait la tour, papa ?
+papa|Tu veux la tour, Mila ?
+enfant-f|Oui, une tour.
+narrateur|Les cubes tapent le bois.
+enfant-f|C'est dur, papa.
+papa|Comme une maison ?
+enfant-f|Oui, comme une maison.
+narrateur|En ce moment, Mila tire le panier vers le bois.
+enfant-f|Je veux la tour, maintenant !
+enfant-f|La tour, tout de suite.
+papa|Tu vois les cubes, Mila ?
+enfant-f|Oui, papa.
+narrateur|Mila pose un cube, trop vite.
+narrateur|Puis un autre, trop haut.
 narrateur|Les cubes glissent.
 narrateur|La tour tombe.
-narrateur|Les épaules de Sarah se serrent.
-narrateur|Sa poitrine va trop vite.
-enfant-f|C'est trop. Je suis fâchée.
-maman|La tour est tombée. Tu es fâchée.
-maman|On peut souffler.
-papa|On peut faire une pause.
-narrateur|Sarah s'assoit sur le tapis.
-narrateur|Elle pose les mains sur ses genoux.
-narrateur|Elle souffle une fois.
-narrateur|Elle souffle encore.
-narrateur|Elle fait une pause.
-narrateur|La pause dure un moment.
-narrateur|La lampe reste ronde et calme.
-enfant-f|Je souffle. Je fais une pause.
-maman|Bravo. Tes épaules redescendent.
-papa|Tu as soufflé. Tu as fait une pause.
-maman|Tu veux reprendre, tout doucement ?
-enfant-f|Oui. Un cube, puis un autre.
-narrateur|Sarah reprend les cubes.
-narrateur|Elle pose un cube, puis un autre.
-narrateur|La tour tient.</t>
+enfant-f|Oh.
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules se serrent.
+papa|Elle est tombée, Mila ?
+enfant-f|Oui, papa.
+maman|Tes lèvres sont serrées, Mila ?
+enfant-f|Un peu, maman.
+narrateur|L'éclat d'étagère tremble, puis tient.
+narrateur|Les cubes restent au sol, mêlés.
+enfant-f|C'est trop, maman.
+narrateur|Maman s'accroupit à la même hauteur.
+narrateur|Mila regarde maman.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1398,17 +1417,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>La tour de Sarah tombe. Que fait-elle ?</t>
+          <t>La tour de Mila tombe. Que fait-elle ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>La tour de Sarah tombe. Que fait-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;La tour de &lt;emphasis level="moderate"&gt;Mila&lt;/emphasis&gt; tombe. Que fait-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>La tour de Flore tombe. Que fait-elle ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;La tour de &lt;emphasis&gt;Mila&lt;/emphasis&gt; tombe. Que fait-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1433,7 +1452,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Elle s'assoit. Elle souffle. Elle fait une pause. Que fait Flore ?</t>
+          <t>Elle s'assoit. Elle souffle. Elle fait une pause. Que fait Mila ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1471,18 +1490,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1497,34 +1516,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Mila</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1533,28 +1556,28 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=la_tour_tombe_que_fait_elle; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|La tour de Sarah tombe.
+          <t>narrateur|La tour de Mila tombe.
 narrateur|Que fait-elle ?</t>
         </is>
       </c>
@@ -1582,17 +1605,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sarah a soufflé. Elle a fait une pause. Elle s'est assise. Puis elle a repris. Le verre d'eau est là, si tu veux. Plus tard. D'abord le puzzle. La boîte est ouverte. On peut essayer. Plus tard, elle ouvre le puzzle. Les pièces sont lisses et un peu froides. Une pièce résiste. Sarah sent encore ses épaules. Je me souviens. Je souffle. Je fais une pause. Oui. Tu t'assois. Tu souffles. La pause aide. Ensuite on reprend. Sarah s'assoit. Elle souffle. Elle fait une pause. Ensuite elle reprend une pièce. La pièce entre. Bravo. J'ai soufflé. C'est plus calme.</t>
+          <t>Mila veut la tour, tout de suite. Je construis, maintenant ! Elle avance trop vite vers les cubes. Un cube bascule. Mila baisse les yeux. Sa poitrine est coincée. C'est trop. Mila s'assoit près du bois. Elle souffle une fois. Elle souffle, plus long. Ses mains se posent sur ses genoux. Personne ne parle. Elle observe l'étagère, un instant. Elle écoute le silence de la chambre. Tu veux la tour, Mila ? Papa reste à la même hauteur. Papa, on fait quoi ? On laisse un peu d'air ? D'accord. Mila reste un moment, sans bouger. Ses épaules redescendent. Le bois est tiède, sous les doigts. Il est chaud. Merci, Mila. Papa a vu les deux, dans la chambre. Mila reprend un cube. Elle le pose, sans se presser. La tour. Elle a un toit, là ? Oui, là. Mila glisse la main près du panier. Le bois est lisse, contre la peau. Tes mains sont au chaud, Mila ? Un peu, maman. Papa s'assoit, puis se relève. On la pose au bord ? La tour va jusqu'à l'étagère. Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sarah a soufflé. Elle a fait une pause. Elle s'est assise. Puis elle a repris. Le verre d'eau est là, si tu veux. Plus tard. D'abord le puzzle. La boîte est ouverte. On peut essayer. Plus tard, elle ouvre le puzzle. Les pièces sont lisses et un peu froides. Une pièce résiste. Sarah sent encore ses épaules. Je me souviens. Je souffle. Je fais une pause. Oui. Tu t'assois. Tu souffles. La pause aide. Ensuite on reprend. Sarah s'assoit. Elle souffle. Elle fait une pause. Ensuite elle reprend une pièce. La pièce entre. Bravo. J'ai soufflé. C'est plus calme.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila veut la tour, tout de suite. Je construis, maintenant ! Elle avance trop vite vers les cubes. Un cube bascule. Mila baisse les yeux. Sa poitrine est coincée. C'est trop. Mila s'assoit près du bois. Elle &lt;emphasis level="moderate"&gt;souffle&lt;/emphasis&gt; une fois. Elle souffle, plus long. Ses mains se posent sur ses genoux. Personne ne parle. Elle observe l'étagère, un instant. Elle écoute le silence de la chambre. Tu veux la tour, Mila ? Papa reste à la même hauteur. Papa, on fait quoi ? On laisse un peu d'air ? D'accord. Mila reste un moment, sans bouger. Ses épaules redescendent. Le bois est tiède, sous les doigts. Il est chaud. Merci, Mila. Papa a vu les deux, dans la chambre. Mila reprend un cube. Elle le pose, sans se presser. La tour. Elle a un toit, là ? Oui, là. Mila glisse la main près du panier. Le bois est lisse, contre la peau. Tes mains sont au chaud, Mila ? Un peu, maman. Papa s'assoit, puis se relève. On la pose au bord ? La tour va jusqu'à l'étagère. Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Flore a soufflé. Elle a fait une &lt;emphasis&gt;pause&lt;/emphasis&gt;. Elle s'est assise. Puis elle a repris. [pause]</t>
+          <t>Mila veut la tour, tout de suite. Je construis, maintenant ! Elle avance trop vite vers les cubes. Un cube bascule. Mila baisse les yeux. Sa poitrine est coincée. C'est trop. Mila s'assoit près du bois. Elle &lt;emphasis&gt;souffle&lt;/emphasis&gt; une fois. Elle souffle, plus long. Ses mains se posent sur ses genoux. Personne ne parle. Elle observe l'étagère, un instant. Elle écoute le silence de la chambre. Tu veux la tour, Mila ? Papa reste à la même hauteur. Papa, on fait quoi ? On laisse un peu d'air ? D'accord. Mila reste un moment, sans bouger. Ses épaules redescendent. Le bois est tiède, sous les doigts. Il est chaud. Merci, Mila. Papa a vu les deux, dans la chambre. Mila reprend un cube. Elle le pose, sans se presser. La tour. Elle a un toit, là ? Oui, là. Mila glisse la main près du panier. Le bois est lisse, contre la peau. Tes mains sont au chaud, Mila ? Un peu, maman. Papa s'assoit, puis se relève. On la pose au bord ? La tour va jusqu'à l'étagère. Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1639,7 +1662,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1647,10 +1670,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1673,30 +1696,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>pause</t>
+          <t>souffle</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1705,10 +1728,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1721,35 +1744,54 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=gêne puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_souffle_elle_reste; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sarah a soufflé.
-narrateur|Elle a fait une pause.
-narrateur|Elle s'est assise. Puis elle a repris.
-papa|Le verre d'eau est là, si tu veux.
-enfant-f|Plus tard. D'abord le puzzle.
-maman|La boîte est ouverte. On peut essayer.
-narrateur|Plus tard, elle ouvre le puzzle.
-narrateur|Les pièces sont lisses et un peu froides.
-narrateur|Une pièce résiste.
-narrateur|Sarah sent encore ses épaules.
-enfant-f|Je me souviens. Je souffle. Je fais une pause.
-papa|Oui. Tu t'assois. Tu souffles.
-maman|La pause aide. Ensuite on reprend.
-narrateur|Sarah s'assoit.
-narrateur|Elle souffle.
-narrateur|Elle fait une pause.
-narrateur|Ensuite elle reprend une pièce.
-papa|La pièce entre. Bravo.
-enfant-f|J'ai soufflé. C'est plus calme.</t>
+          <t>narrateur|Mila veut la tour, tout de suite.
+enfant-f|Je construis, maintenant !
+narrateur|Elle avance trop vite vers les cubes.
+narrateur|Un cube bascule.
+narrateur|Mila baisse les yeux.
+narrateur|Sa poitrine est coincée.
+enfant-f|C'est trop.
+narrateur|Mila s'assoit près du bois.
+narrateur|Elle souffle une fois.
+narrateur|Elle souffle, plus long.
+narrateur|Ses mains se posent sur ses genoux.
+narrateur|Personne ne parle.
+narrateur|Elle observe l'étagère, un instant.
+narrateur|Elle écoute le silence de la chambre.
+papa|Tu veux la tour, Mila ?
+narrateur|Papa reste à la même hauteur.
+enfant-f|Papa, on fait quoi ?
+papa|On laisse un peu d'air ?
+enfant-f|D'accord.
+narrateur|Mila reste un moment, sans bouger.
+narrateur|Ses épaules redescendent.
+maman|Le bois est tiède, sous les doigts.
+enfant-f|Il est chaud.
+papa|Merci, Mila.
+narrateur|Papa a vu les deux, dans la chambre.
+narrateur|Mila reprend un cube.
+narrateur|Elle le pose, sans se presser.
+enfant-f|La tour.
+maman|Elle a un toit, là ?
+enfant-f|Oui, là.
+narrateur|Mila glisse la main près du panier.
+narrateur|Le bois est lisse, contre la peau.
+maman|Tes mains sont au chaud, Mila ?
+enfant-f|Un peu, maman.
+narrateur|Papa s'assoit, puis se relève.
+enfant-f|On la pose au bord ?
+maman|La tour va jusqu'à l'étagère.
+enfant-f|Oui, maman.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>puzzle</t>
+          <t>cubes</t>
         </is>
       </c>
     </row>
@@ -1776,17 +1818,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sarah range un cube dans le panier. Le verre d'eau fait un petit bruit. Tu veux une gorgée ? Oui, papa. Tu as fini la petite tour ? Oui. Et une pièce du puzzle. Tu as soufflé. Tu as fait une pause. Les chaussettes sont sèches. La lampe ronde veille encore.</t>
+          <t>Ils restent près de l'étagère. La tour penche d'un côté. Le toit, maintenant ! Mila tire un cube trop vite. Le cube part derrière l'étagère. Je ne le vois plus ! Elle se penche, trop vite. La tour tremble, cette fois. Oh ! Mila s'arrête net. Elle souffle, un filet d'air. Elle reste un moment, les mains ouvertes. Personne ne dit la suite. Elle observe le bord, un instant. Elle écoute le silence de la chambre. Au bord du bois, un éclat d'étagère luit. Là, sur le bois. Le cube est derrière, papa ? Tu le vois, derrière l'étagère ? Oui, papa. Mila prend le cube, sans se presser. Elle le pose sur la tour. Le bois est lisse et tiède. Tu le vois, le bord ? Oui, maman. La tour est près de l'étagère ? Oui, papa. Mila pose un cube. Papa pose une main sur le bois. La tour tient, Mila ? Oui, maman. Un rayon passe sur l'étagère. Il allume le bois.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sarah range un cube dans le panier. Le verre d'eau fait un petit bruit. Tu veux une gorgée ? Oui, papa. Tu as fini la petite tour ? Oui. Et une pièce du puzzle. Tu as soufflé. Tu as fait une pause. Les chaussettes sont sèches. La lampe ronde veille encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils restent près de l'étagère. La tour penche d'un côté. Le toit, maintenant ! Mila tire un cube trop vite. Le cube part derrière l'étagère. Je ne le vois plus ! Elle se penche, trop vite. La tour tremble, cette fois. Oh ! Mila s'arrête net. Elle souffle, un filet d'air. Elle reste un moment, les mains ouvertes. Personne ne dit la suite. Elle observe le bord, un instant. Elle écoute le silence de la chambre. Au bord du bois, un &lt;emphasis level="moderate"&gt;éclat d'étagère&lt;/emphasis&gt; luit. Là, sur le bois. Le cube est derrière, papa ? Tu le vois, derrière l'étagère ? Oui, papa. Mila prend le cube, sans se presser. Elle le pose sur la tour. Le bois est lisse et tiède. Tu le vois, le bord ? Oui, maman. La tour est près de l'étagère ? Oui, papa. Mila pose un cube. Papa pose une main sur le bois. La tour tient, Mila ? Oui, maman. Un rayon passe sur l'étagère. Il allume le bois.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Flore range un cube. Maman lui tend la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Ils restent près de l'étagère. La tour penche d'un côté. Le toit, maintenant ! Mila tire un cube trop vite. Le cube part derrière l'étagère. Je ne le vois plus ! Elle se penche, trop vite. La tour tremble, cette fois. Oh ! Mila s'arrête net. Elle souffle, un filet d'air. Elle reste un moment, les mains ouvertes. Personne ne dit la suite. Elle observe le bord, un instant. Elle écoute le silence de la chambre. Au bord du bois, un &lt;emphasis&gt;éclat d'étagère&lt;/emphasis&gt; luit. Là, sur le bois. Le cube est derrière, papa ? Tu le vois, derrière l'étagère ? Oui, papa. Mila prend le cube, sans se presser. Elle le pose sur la tour. Le bois est lisse et tiède. Tu le vois, le bord ? Oui, maman. La tour est près de l'étagère ? Oui, papa. Mila pose un cube. Papa pose une main sur le bois. La tour tient, Mila ? Oui, maman. Un rayon passe sur l'étagère. Il allume le bois. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1833,7 +1875,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1841,10 +1883,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1867,30 +1909,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat d'étagère</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1899,10 +1941,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1913,23 +1955,51 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=cube_derriere_etagere_elle_souffle; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Sarah range un cube dans le panier.
-narrateur|Le verre d'eau fait un petit bruit.
-papa|Tu veux une gorgée ?
+          <t>narrateur|Ils restent près de l'étagère.
+narrateur|La tour penche d'un côté.
+enfant-f|Le toit, maintenant !
+narrateur|Mila tire un cube trop vite.
+narrateur|Le cube part derrière l'étagère.
+enfant-f|Je ne le vois plus !
+narrateur|Elle se penche, trop vite.
+narrateur|La tour tremble, cette fois.
+enfant-f|Oh !
+narrateur|Mila s'arrête net.
+narrateur|Elle souffle, un filet d'air.
+narrateur|Elle reste un moment, les mains ouvertes.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe le bord, un instant.
+narrateur|Elle écoute le silence de la chambre.
+narrateur|Au bord du bois, un éclat d'étagère luit.
+enfant-f|Là, sur le bois.
+enfant-f|Le cube est derrière, papa ?
+papa|Tu le vois, derrière l'étagère ?
 enfant-f|Oui, papa.
-maman|Tu as fini la petite tour ?
-enfant-f|Oui. Et une pièce du puzzle.
-maman|Tu as soufflé. Tu as fait une pause.
-narrateur|Les chaussettes sont sèches.
-narrateur|La lampe ronde veille encore.</t>
+narrateur|Mila prend le cube, sans se presser.
+narrateur|Elle le pose sur la tour.
+narrateur|Le bois est lisse et tiède.
+maman|Tu le vois, le bord ?
+enfant-f|Oui, maman.
+papa|La tour est près de l'étagère ?
+enfant-f|Oui, papa.
+narrateur|Mila pose un cube.
+narrateur|Papa pose une main sur le bois.
+maman|La tour tient, Mila ?
+enfant-f|Oui, maman.
+papa|Un rayon passe sur l'étagère.
+enfant-f|Il allume le bois.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>verre_eau</t>
+          <t>cubes</t>
         </is>
       </c>
     </row>
@@ -1956,17 +2026,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai soufflé. J'ai fait une pause. Bravo, Sarah. La tour tient. Le puzzle attend demain.</t>
+          <t>Ils restent près de l'étagère. La tour est arrivée, Mila ? Oui, maman. Tu souffles un peu ? Oui, papa. Mila souffle, un filet d'air. Le bois sent la cire. Tu le sens, le bois ? Oui, maman. La tour reste un peu, de travers. Elle a tenu, sur le bois. Le bois est chaud, sous les mains. L'étagère fait une petite ombre. On y retourne, après. Un éclat d'étagère tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai soufflé. J'ai fait une pause. Bravo, Sarah. La tour tient. Le puzzle attend demain.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de l'étagère. La tour est arrivée, Mila ? Oui, maman. Tu souffles un peu ? Oui, papa. Mila souffle, un filet d'air. Le bois sent la cire. Tu le sens, le bois ? Oui, maman. La tour reste un peu, de travers. Elle a tenu, sur le bois. Le bois est chaud, sous les mains. L'étagère fait une petite ombre. On y retourne, après. Un &lt;emphasis level="moderate"&gt;éclat d'étagère&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de l'étagère. La tour est arrivée, Mila ? Oui, maman. Tu souffles un peu ? Oui, papa. Mila souffle, un filet d'air. Le bois sent la cire. Tu le sens, le bois ? Oui, maman. La tour reste un peu, de travers. Elle a tenu, sur le bois. Le bois est chaud, sous les mains. L'étagère fait une petite ombre. On y retourne, après. Un &lt;emphasis&gt;éclat d'étagère&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2013,18 +2083,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2033,12 +2103,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2047,17 +2117,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat d'étagère</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2066,11 +2140,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2079,26 +2153,42 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai soufflé. J'ai fait une pause.
-maman|Bravo, Sarah.
-papa|La tour tient. Le puzzle attend demain.</t>
+          <t>narrateur|Ils restent près de l'étagère.
+maman|La tour est arrivée, Mila ?
+enfant-f|Oui, maman.
+papa|Tu souffles un peu ?
+enfant-f|Oui, papa.
+narrateur|Mila souffle, un filet d'air.
+enfant-f|Le bois sent la cire.
+maman|Tu le sens, le bois ?
+enfant-f|Oui, maman.
+papa|La tour reste un peu, de travers.
+enfant-f|Elle a tenu, sur le bois.
+narrateur|Le bois est chaud, sous les mains.
+narrateur|L'étagère fait une petite ombre.
+enfant-f|On y retourne, après.
+narrateur|Un éclat d'étagère tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2209,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2183,6 +2273,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>